<commit_message>
feat - adicionado front visual com streamlit
</commit_message>
<xml_diff>
--- a/relatorio_nfe.xlsx
+++ b/relatorio_nfe.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -591,6 +591,356 @@
       <c r="G5" t="inlineStr">
         <is>
           <t>02/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>35250214200166000187550010000000051000000051</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1005</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2025-02-25</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>14200166000187</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Distribuidora Sertao Ltda</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>1200</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>02/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>35250314200166000187550010000000061000000062</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1006</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2025-03-03</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>09876543000122</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Atacado Garanhuns ME</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>3450.9</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>03/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>35250314200166000187550010000000071000000073</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1007</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2025-03-12</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>55667788000199</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Mercado Caruaru Ltda</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>780.45</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>03/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>35250314200166000187550010000000081000000084</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1008</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2025-03-20</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>33444555000166</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Comercial Agreste SA</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>5600</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>03/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>35250314200166000187550010000000091000000095</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1009</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2025-03-28</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>14200166000187</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Distribuidora Sertao Ltda</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>920.3</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>03/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>35250414200166000187550010000000101000000106</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1010</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2025-04-05</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>55667788000199</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Mercado Caruaru Ltda</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>35250414200166000187550010000000111000000117</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>1011</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2025-04-15</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>09876543000122</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Atacado Garanhuns ME</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>467.8</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>35250414200166000187550010000000121000000128</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>1012</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2025-04-22</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>77888999000111</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Distribuidora Recife SA</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>8900.5</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>04/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>35250514200166000187550010000000131000000139</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>1013</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2025-05-02</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>33444555000166</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Comercial Agreste SA</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>1340</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>05/2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>35250514200166000187550010000000141000000140</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>1014</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2025-05-18</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>77888999000111</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Distribuidora Recife SA</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>3275.65</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>05/2025</t>
         </is>
       </c>
     </row>
@@ -605,7 +955,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -637,7 +987,37 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2760.95</v>
+        <v>3960.95</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>03/2025</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>10751.65</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>04/2025</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>11468.3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>05/2025</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>4615.65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>